<commit_message>
all the changes today
</commit_message>
<xml_diff>
--- a/projects/neuronal_migration_analysis/data/Analysis R3/Tron Intermediate files/control/10x_1024_1umZ_KC63_M1_shc202_section_B_cropgreen ANALYSIS.xlsx
+++ b/projects/neuronal_migration_analysis/data/Analysis R3/Tron Intermediate files/control/10x_1024_1umZ_KC63_M1_shc202_section_B_cropgreen ANALYSIS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ciziok\Desktop\Temporary File Location\Analysis\10x_1024_1umZ_KC63_M1_shc202_section_B_cropgreen 27-01-2025 15-57-47\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ciziok\katcizio.github.io\projects\neuronal_migration_analysis\data\Analysis R3\Tron Intermediate files\control\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2035B51-3D78-45B5-96ED-BA80E952BF6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8474F369-78CE-476F-B1EB-E354BDFA4642}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1185" yWindow="3060" windowWidth="34320" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Green" sheetId="1" r:id="rId1"/>
@@ -438,13 +438,14 @@
   <dimension ref="A1:H271"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="48.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="47.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>